<commit_message>
further additions to JS and CSS
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/content/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71FBF8B-7C26-774B-A389-7FE3DA0E76B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFF456F-DEBA-B74F-A90E-5EF9A8F44AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="560" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
   <sheets>
     <sheet name="timeline" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="96">
   <si>
     <t>class</t>
   </si>
@@ -282,6 +282,48 @@
   </si>
   <si>
     <t>timeline-1 time-travel event</t>
+  </si>
+  <si>
+    <t>The Nobleman Kain departs from his home city of Coorhagen on a journey across Nosgoth. During his travel Kain is ambushed by brigands, who murder and cruelly impale him with a sword.</t>
+  </si>
+  <si>
+    <t>Events of Blood Omen: Legacy of Kain</t>
+  </si>
+  <si>
+    <t>Kain's body is interred in a crypt west of Ziegsturhl.</t>
+  </si>
+  <si>
+    <t>Kain awakens in the underworld, where Mortanius offers to revive him, so that Kain may take revenge upon his assassins. Kain, heedless of the cost, accepts the necromancer's offer. The catch: in order to rejoin the world of the living, Kain is reborn as a vampire.</t>
+  </si>
+  <si>
+    <t>Kain awakens in his mausoleum, and begins his "unlife" as a vampire.</t>
+  </si>
+  <si>
+    <t>timeline-1 game</t>
+  </si>
+  <si>
+    <t>Kain finds his assassins and kills them, getting his revenge - but Mortanius drives him on to the Pillars, saying that the brigands were only the instruments of his murder, not the cause.</t>
+  </si>
+  <si>
+    <t>Kain hunts down and destroys the corrupt Circle Guardians, restoring each of the Pillars in turn</t>
+  </si>
+  <si>
+    <t>Kain meets the ancient vampire Vorador</t>
+  </si>
+  <si>
+    <t>Kain discovers the &lt;b&gt;Soul Reaver&lt;/b&gt; within Avernus Cathedral, and claims it for his own</t>
+  </si>
+  <si>
+    <t>Ariel warns Kain of the impending assault from the Nemesis armies to the north, and that Willendorf is next in their path. She tells him of the Nemesis, how this tyrant was once William the Just, a kind and benevolent king.</t>
+  </si>
+  <si>
+    <t>The Armies of Hope are decimated; Kain activates the Time Streaming Device, and is propelled nearly 50 years back in time</t>
+  </si>
+  <si>
+    <t>Kain confronts and defeats the planer Azimuth. He also discovers a mysterious Time Streaming Device, which Azimuth has apparently stolen from Moebius (the Guardian of Time).</t>
+  </si>
+  <si>
+    <t>#travel-1</t>
   </si>
 </sst>
 </file>
@@ -696,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -1322,6 +1364,144 @@
         <v>57</v>
       </c>
     </row>
+    <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E68" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I68" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I69" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I70" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I71" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I73" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A74" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I74" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A75" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I75" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I76" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A77" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="I79" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
scrolling issue now resolved
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFF456F-DEBA-B74F-A90E-5EF9A8F44AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA95F7B-8E92-0047-BA76-227C46B69A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="97">
   <si>
     <t>class</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Ariel's murder drives her beloved, Nupraptor (the Pillar of the Mind), insane with grief. In his agony, he unleashes a telepathic assault which ripples across the Land of Nosgoth, infecting the other members of the Circle (who are all symbiotically connected) with his madness.</t>
   </si>
   <si>
-    <t>timeline-1 time-travel tt1 event</t>
-  </si>
-  <si>
     <t>Human Raziel is born, and becomes a Sarafan warrior-priest</t>
   </si>
   <si>
@@ -324,6 +321,12 @@
   </si>
   <si>
     <t>#travel-1</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel travel-1</t>
+  </si>
+  <si>
+    <t>BloodOmen</t>
   </si>
 </sst>
 </file>
@@ -947,7 +950,7 @@
         <v>5</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -966,7 +969,7 @@
         <v>5</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -974,7 +977,7 @@
         <v>5</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -993,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1001,7 +1004,7 @@
         <v>5</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1009,7 +1012,7 @@
         <v>5</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1017,7 +1020,7 @@
         <v>5</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1025,7 +1028,7 @@
         <v>5</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1033,7 +1036,7 @@
         <v>5</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1041,7 +1044,7 @@
         <v>5</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1049,7 +1052,7 @@
         <v>5</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1060,12 +1063,12 @@
         <v>1</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="I34" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1073,7 +1076,7 @@
         <v>26</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1081,7 +1084,7 @@
         <v>5</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1097,7 +1100,7 @@
         <v>5</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1188,7 +1191,7 @@
         <v>5</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1196,12 +1199,12 @@
         <v>5</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>40</v>
@@ -1210,62 +1213,62 @@
         <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>48</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B53" t="s">
         <v>48</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B54" t="s">
         <v>48</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B55" t="s">
         <v>48</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="56" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B56" t="s">
         <v>48</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="57" spans="1:9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1275,7 +1278,7 @@
     <row r="58" spans="1:9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="60" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>48</v>
@@ -1289,7 +1292,7 @@
     </row>
     <row r="61" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>48</v>
@@ -1361,21 +1364,24 @@
         <v>26</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>48</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>96</v>
       </c>
       <c r="E68" s="3" t="b">
         <v>1</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1386,7 +1392,7 @@
         <v>48</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1397,7 +1403,7 @@
         <v>48</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1408,7 +1414,7 @@
         <v>48</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1419,7 +1425,7 @@
         <v>48</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1430,7 +1436,7 @@
         <v>48</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1441,7 +1447,7 @@
         <v>48</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1452,7 +1458,7 @@
         <v>48</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1463,7 +1469,7 @@
         <v>48</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1474,7 +1480,7 @@
         <v>48</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1485,7 +1491,7 @@
         <v>48</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1496,10 +1502,10 @@
         <v>48</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corrections to newly created timelines before pseudo styles
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA95F7B-8E92-0047-BA76-227C46B69A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92357F95-BAD7-7B43-81B0-234A411799A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
   <si>
     <t>class</t>
   </si>
@@ -1206,6 +1206,9 @@
       <c r="A51" s="3" t="s">
         <v>95</v>
       </c>
+      <c r="B51" t="s">
+        <v>48</v>
+      </c>
       <c r="C51" s="3" t="s">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
further updates to code, starts styling anchors, adds lottie
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92357F95-BAD7-7B43-81B0-234A411799A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E349C0A-5ED5-3D45-A341-4503B154C7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="98">
   <si>
     <t>class</t>
   </si>
@@ -327,6 +327,9 @@
   </si>
   <si>
     <t>BloodOmen</t>
+  </si>
+  <si>
+    <t>Kain confronts William, each of them armed with the Soul Reaver (incarnations of the same weapon at different periods of time). Kain is victorious, and he triumphantly drinks the blood of the fallen king – this is witnessed by the king's guards, come to aid their martyred ruler.</t>
   </si>
 </sst>
 </file>
@@ -741,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -1212,7 +1215,8 @@
       <c r="C51" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D51" t="b">
+      <c r="D51" s="3"/>
+      <c r="E51" t="b">
         <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
@@ -1241,27 +1245,23 @@
         <v>76</v>
       </c>
     </row>
-    <row r="54" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B54" t="s">
-        <v>48</v>
+      <c r="B54" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G54" s="3" t="b">
+        <v>1</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B55" t="s">
-        <v>48</v>
-      </c>
-      <c r="I55" s="4" t="s">
-        <v>79</v>
-      </c>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="3"/>
+      <c r="I55" s="4"/>
     </row>
     <row r="56" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
@@ -1271,87 +1271,87 @@
         <v>48</v>
       </c>
       <c r="I56" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B57" t="s">
+        <v>48</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A58" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B58" t="s">
+        <v>48</v>
+      </c>
+      <c r="I58" s="4" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="57" spans="1:9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="3"/>
-      <c r="I57" s="4"/>
-    </row>
-    <row r="58" spans="1:9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I60" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I61" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
+    <row r="59" spans="1:9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="3"/>
+      <c r="I59" s="4"/>
+    </row>
+    <row r="60" spans="1:9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="62" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D63" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I63" s="2" t="s">
-        <v>51</v>
+        <v>80</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B65" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I65" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="E65" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>5</v>
       </c>
@@ -1359,54 +1359,54 @@
         <v>48</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I67" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I68" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I67" s="4" t="s">
+      <c r="I69" s="4" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E68" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I68" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I69" s="4" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
-        <v>5</v>
+        <v>86</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>48</v>
       </c>
+      <c r="C70" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D70" s="3" t="b">
+        <v>1</v>
+      </c>
       <c r="I70" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1417,7 +1417,7 @@
         <v>48</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1428,7 +1428,7 @@
         <v>48</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1439,7 +1439,7 @@
         <v>48</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1450,10 +1450,10 @@
         <v>48</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>5</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>48</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1472,42 +1472,64 @@
         <v>48</v>
       </c>
       <c r="I76" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I78" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A77" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I77" s="4" t="s">
+    <row r="79" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I79" s="4" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A78" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I78" s="4" t="s">
+    <row r="80" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I80" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F79" s="3" t="s">
+    <row r="81" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F81" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="I79" s="4" t="s">
+      <c r="I81" s="4" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
starts dealing with paradoxes
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E349C0A-5ED5-3D45-A341-4503B154C7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E0D5AA-B9F1-7F4E-8503-CD9B816ECDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
   <si>
     <t>class</t>
   </si>
@@ -161,15 +161,9 @@
     <t>travel-1</t>
   </si>
   <si>
-    <t>Kain assassinates the young King William the Just, who will become the Nemesis</t>
-  </si>
-  <si>
     <t>#paradox-1</t>
   </si>
   <si>
-    <t>Kain discovers another Time Streaming Device and returns to Nosgoth's present</t>
-  </si>
-  <si>
     <t>#travel-2</t>
   </si>
   <si>
@@ -278,9 +272,6 @@
     <t>Devastated by William's murder at the hands of a vampire, the people of William's realm swear a vengeful covenant to their fallen king, promising to eradicate Nosgoth's vampires once and for all.</t>
   </si>
   <si>
-    <t>timeline-1 time-travel event</t>
-  </si>
-  <si>
     <t>The Nobleman Kain departs from his home city of Coorhagen on a journey across Nosgoth. During his travel Kain is ambushed by brigands, who murder and cruelly impale him with a sword.</t>
   </si>
   <si>
@@ -330,6 +321,12 @@
   </si>
   <si>
     <t>Kain confronts William, each of them armed with the Soul Reaver (incarnations of the same weapon at different periods of time). Kain is victorious, and he triumphantly drinks the blood of the fallen king – this is witnessed by the king's guards, come to aid their martyred ruler.</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel paradox-1</t>
+  </si>
+  <si>
+    <t>Kain discovers the Time Streaming Device and escapes back into the future – secure in his belief that he has thwarted Moebius's machinations by removing his pawn William from the game.</t>
   </si>
 </sst>
 </file>
@@ -744,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -759,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>39</v>
@@ -953,7 +950,7 @@
         <v>5</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -972,7 +969,7 @@
         <v>5</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -980,7 +977,7 @@
         <v>5</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -999,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1007,7 +1004,7 @@
         <v>5</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1015,7 +1012,7 @@
         <v>5</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1023,7 +1020,7 @@
         <v>5</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1031,7 +1028,7 @@
         <v>5</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1039,7 +1036,7 @@
         <v>5</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1047,7 +1044,7 @@
         <v>5</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1055,7 +1052,7 @@
         <v>5</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1066,12 +1063,12 @@
         <v>1</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="I34" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1079,7 +1076,7 @@
         <v>26</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1087,7 +1084,7 @@
         <v>5</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1103,7 +1100,7 @@
         <v>5</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1130,7 +1127,7 @@
         <v>5</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1189,174 +1186,175 @@
         <v>38</v>
       </c>
     </row>
-    <row r="49" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>5</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>5</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B51" t="s">
-        <v>48</v>
+        <v>92</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D51" s="3"/>
-      <c r="E51" t="b">
+      <c r="E51" s="3" t="b">
         <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A54" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B52" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I52" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B53" t="s">
-        <v>48</v>
-      </c>
-      <c r="I53" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A54" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G54" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="3"/>
-      <c r="I55" s="4"/>
-    </row>
-    <row r="56" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B55" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B56" t="s">
-        <v>48</v>
+      <c r="B56" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B57" t="s">
-        <v>48</v>
+      <c r="B57" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B58" t="s">
-        <v>48</v>
+      <c r="B58" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="3"/>
-      <c r="I59" s="4"/>
-    </row>
-    <row r="60" spans="1:9" customFormat="1" x14ac:dyDescent="0.2"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I60" s="3"/>
+    </row>
     <row r="62" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I63" s="4" t="s">
-        <v>43</v>
+        <v>5</v>
+      </c>
+      <c r="E63" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E65" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I65" s="2" t="s">
+      <c r="B65" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I65" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>52</v>
@@ -1364,49 +1362,49 @@
     </row>
     <row r="67" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D68" s="3" t="b">
+        <v>1</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>26</v>
+        <v>5</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
-        <v>86</v>
+        <v>5</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D70" s="3" t="b">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1414,7 +1412,7 @@
         <v>5</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>81</v>
@@ -1425,10 +1423,10 @@
         <v>5</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1436,7 +1434,7 @@
         <v>5</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>84</v>
@@ -1447,21 +1445,21 @@
         <v>5</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1469,68 +1467,46 @@
         <v>5</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I76" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A77" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I78" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A77" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I77" s="4" t="s">
+    <row r="79" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I79" s="4" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A78" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I78" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I79" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A80" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I80" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A81" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I81" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
small additions to styles
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C40AD01-7572-CF4A-A9BF-F7B16DCAF56E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA1DA7CA-CAF2-EC48-AF78-C732DA8FA50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="109">
   <si>
     <t>class</t>
   </si>
@@ -330,6 +330,39 @@
   </si>
   <si>
     <t>paradox-1</t>
+  </si>
+  <si>
+    <t>Upon returning to the future, however, Kain discovers that his actions have dramatically altered the course of Nosgoth's history. The assassination of  William triggered a renewed vampire purge. The Nemesis has now never existed.</t>
+  </si>
+  <si>
+    <t>Kain confronts and kills Moebius, the Guardian of Time.</t>
+  </si>
+  <si>
+    <t>Vorador is executed by Moebius and his Vampire Hunters; Kain is the only surviving vampire in Nosgoth.</t>
+  </si>
+  <si>
+    <t>travel-2</t>
+  </si>
+  <si>
+    <t>The Dark Entity possessing Mortanius taunts Kain, saying that Kain has been no more than a pawn, and that all of the preceding events have been orchestrated from the beginning. Kain launches himself at the Dark Entity, and using the Soul Reaver, manages to defeat him. It's not clear, however, whether the Dark Entity has been destroyed or merely dispelled</t>
+  </si>
+  <si>
+    <t>The Collapse of the Pillars</t>
+  </si>
+  <si>
+    <t>Ariel appears and reveals to Kain that he himself is the Pillar of Balance, and that the only way the Pillars can be healed is for him to sacrifice himself – as the last of the Circle – to the Pillar. She presents him with the final, climactic decision — sacrifice himself to heal the world, or refuse the sacrifice and ensure the world's corruption.</t>
+  </si>
+  <si>
+    <t>Kain chooses the latter path, deciding to rule the world in its damnation rather than commit himself to oblivion. This apocalyptic act completes the Pillars' destruction – the Pillars topple as Kain seals their ruinous fate.</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel travel-1 detail</t>
+  </si>
+  <si>
+    <t>Roughly 500 years after Blood Omen: Legacy of Kain</t>
+  </si>
+  <si>
+    <t>The raising of the lieutenants</t>
   </si>
 </sst>
 </file>
@@ -744,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -1515,6 +1548,108 @@
         <v>89</v>
       </c>
     </row>
+    <row r="80" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="I80" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I81" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A82" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I82" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A83" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I83" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E84" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I84" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I85" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I86" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="I87" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A88" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E88" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I88" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
more updates to content and styles
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1F4E6A-8BE2-A749-86F9-D0AB6DD1D5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7DDDBB-68D4-8947-B03D-1186241F0375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="127">
   <si>
     <t>class</t>
   </si>
@@ -366,6 +366,57 @@
   </si>
   <si>
     <t>Kain sets the ruined Pillars as the seat of his new empire and the unresored Balance Pillar as the base of his throne.</t>
+  </si>
+  <si>
+    <t>Kain raises his six vampire lieutenants from the corpses of the Sarafan martyrs using ancient Necromancing techinques - each lieutenant is raised using a Pillar element; Raziel is reborn as a vampire.</t>
+  </si>
+  <si>
+    <t>Kain's empire grows. The six lieutenants recruit clans of their own, "turning" the corpses of their human victims to do their bidding.</t>
+  </si>
+  <si>
+    <t>The destruction of the major human Kingdoms is inevitable. Within a hundred years, humanity is thoroughly domesticated. Some feral humans remain scattered across the hinterlands, clinging to their hopeless holy war to rid Nosgoth of 'the vampire scourge'. They are tolerated. They make existence for the fledglings more challenging.</t>
+  </si>
+  <si>
+    <t>After the taming of the humans, the vampires' real work begins; shaping Nosgoth to their will. Around the Pillars, slaves construct a shrine worthy of their new age and renaissance. Huge furnaces are built to belch smoke into the sky, shielding the land from the poisonous effects of the sun.</t>
+  </si>
+  <si>
+    <t>The lieutenants allow the remains of the legions, the lesser vampires, to have their intrigues. They provide amusement and spice to an increasingly uninspired court. As faction falls against faction they bet upon the outcome. They help and foil plots at their whim. They are the Council and Lord Kain, their only master.</t>
+  </si>
+  <si>
+    <t>Roughly 1500 years after Blood Omen: Legacy of Kain</t>
+  </si>
+  <si>
+    <t>SR</t>
+  </si>
+  <si>
+    <t>SoulReaver</t>
+  </si>
+  <si>
+    <t>Events of Legacy of Kain: Soul Reaver</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel travel-1 game</t>
+  </si>
+  <si>
+    <t>Over the centuries, each of the vampires undergoes a series of evolutionary adaptations. These evolutionary "growth spurts" are preceded by a quiescent, near-hibernatory period of retreat, from which the vampire emerges transformed.</t>
+  </si>
+  <si>
+    <t>Raziel emerges from one of these evolutionary hibernations having grown wings. He returns to the Sanctuary of the Clans to present himself to Kain, and reveal his latest gift.</t>
+  </si>
+  <si>
+    <t>Kain, in an apparent act of jealousy, tears the wings from Raziel's back, and orders Raziel to be cast into the Abyss. His motives are unclear, but this is clearly more than just punishment for Raziel's "evolutionary treachery".</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Raziel's resurrection</t>
+  </si>
+  <si>
+    <t>Raziel is revived by the mysterious Elder God at the bottom of the Abyss and is reborn as a reaver of souls.</t>
+  </si>
+  <si>
+    <t>Raziel returns to reap the vampires' apostate souls and take revenge on his vampire brethren and his creator, Kain.</t>
+  </si>
+  <si>
+    <t>Raziel confronts Kain within the ruins of the Pillars Sanctuary; Kain attacks Raziel with the Soul Reaver - the balde is destroyed on impact. Now a wraith blade, the Soul Reaver intertwines with Raziel and becomes his symbiotic weapon.</t>
   </si>
 </sst>
 </file>
@@ -780,7 +831,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -1661,6 +1712,159 @@
         <v>109</v>
       </c>
     </row>
+    <row r="90" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A90" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A91" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A92" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A93" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I93" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A94" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A95" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="I95" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A96" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D96" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I96" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A97" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A98" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I98" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A99" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I99" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A100" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="I100" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A101" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E101" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I101" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A102" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I102" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A103" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I103" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A104" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I104" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
updates paradox json, more content updates
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7DDDBB-68D4-8947-B03D-1186241F0375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322BF69A-D99B-C841-A4EF-651E60EAB39A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -416,7 +416,7 @@
     <t>Raziel returns to reap the vampires' apostate souls and take revenge on his vampire brethren and his creator, Kain.</t>
   </si>
   <si>
-    <t>Raziel confronts Kain within the ruins of the Pillars Sanctuary; Kain attacks Raziel with the Soul Reaver - the balde is destroyed on impact. Now a wraith blade, the Soul Reaver intertwines with Raziel and becomes his symbiotic weapon.</t>
+    <t>Raziel confronts Kain within the ruins of the Pillars Sanctuary; Kain attacks Raziel with the Soul Reaver - the blade is destroyed on impact. Now a wraith blade, the Soul Reaver intertwines with Raziel and becomes his symbiotic weapon.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
further additions to content
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322BF69A-D99B-C841-A4EF-651E60EAB39A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CAF856D-E9A1-5A4F-8140-C6B671534A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="138">
   <si>
     <t>class</t>
   </si>
@@ -167,12 +167,6 @@
     <t>#travel-2</t>
   </si>
   <si>
-    <t>timeline-2a time-travel tt3</t>
-  </si>
-  <si>
-    <t>Raziel arrives to Nosgoth's past and meets Moebius at the Sarafan fortress, now occupied by the Iron Guard, an army that seeks to avenge the Death of William the Just</t>
-  </si>
-  <si>
     <t>entry</t>
   </si>
   <si>
@@ -417,6 +411,45 @@
   </si>
   <si>
     <t>Raziel confronts Kain within the ruins of the Pillars Sanctuary; Kain attacks Raziel with the Soul Reaver - the blade is destroyed on impact. Now a wraith blade, the Soul Reaver intertwines with Raziel and becomes his symbiotic weapon.</t>
+  </si>
+  <si>
+    <t>Raziel discovers a trail leading into the mountains. It winds around, opening onto the entrance of the Oracle’s Cave. Raziel discovers the long-hidden entrance to the Oracle’s chamber.</t>
+  </si>
+  <si>
+    <t>In the depths of Moebius’ time-streaming apparatus, Raziel discovers a series of portals displaying scenes of past and apparently future events. As he descends, passing these various scenes, he reflects on the images confronting him. The images in the portals imply that the events he’s experienced – and those still to come – have all been predestined.</t>
+  </si>
+  <si>
+    <t>After having worked his way down into the depths of Moebius’ complex, he comes across the “heart” of Moebius’ time-streaming device – the Chronoplast room. Kain reveals himself, stepping out from the shadows of the room.</t>
+  </si>
+  <si>
+    <t>Upon emerging from the Chronoplast time portal, Raziel discovers he has been transported nearly two thousand years into Nosgoth's past, to a time roughly 30 years before Kain's resurrection as a vampire... but a decade after Kain's own ill-fated journey into Nosgoth's history, and his assassination of William the Just.</t>
+  </si>
+  <si>
+    <t>He discovers Moebius waiting to meet him on the other side. Raziel is all too aware of Moebius's deceitful reputation, but realizes that they share a common enemy in Kain, and that he may have to consider a careful alliance with the devious Time-Streamer</t>
+  </si>
+  <si>
+    <t>In William's chapel, Raziel discovers the broken Soul Reaver, causing a Reaver-convergence. The Wraith Blade leeches Raziel's soul energy to restore the damaged physical sword. Raziel threatens Moebius with the Soul Reaver, but stays his hand, and leaves the reconstituted weapon behind.</t>
+  </si>
+  <si>
+    <t>Raziel discovers a stained glass window in the Stronghold, depicting the murder of the vampire Janos Audron at the hands of the Sarafan.</t>
+  </si>
+  <si>
+    <t>Events of Legacy of Kain: Soul Reaver 2</t>
+  </si>
+  <si>
+    <t>SoulReaver2</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel travel-2 game</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel travel-2</t>
+  </si>
+  <si>
+    <t>#SoulReaver2</t>
+  </si>
+  <si>
+    <t>Raziel pursues Kain through Moebius's ancient Chronoplast time portal.</t>
   </si>
 </sst>
 </file>
@@ -831,7 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -846,7 +879,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>39</v>
@@ -1040,7 +1073,7 @@
         <v>5</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1059,7 +1092,7 @@
         <v>5</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1067,7 +1100,7 @@
         <v>5</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1086,7 +1119,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1094,7 +1127,7 @@
         <v>5</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1102,7 +1135,7 @@
         <v>5</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1110,7 +1143,7 @@
         <v>5</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1118,7 +1151,7 @@
         <v>5</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1126,7 +1159,7 @@
         <v>5</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1134,7 +1167,7 @@
         <v>5</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1142,7 +1175,7 @@
         <v>5</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1153,12 +1186,12 @@
         <v>1</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="I34" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1166,7 +1199,7 @@
         <v>26</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1174,7 +1207,7 @@
         <v>5</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1190,7 +1223,7 @@
         <v>5</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1217,7 +1250,7 @@
         <v>5</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1281,7 +1314,7 @@
         <v>5</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1289,15 +1322,15 @@
         <v>5</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>40</v>
@@ -1306,129 +1339,165 @@
         <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>41</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>42</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I60" s="3"/>
-    </row>
-    <row r="62" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A59" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D59" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>43</v>
+        <v>135</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>44</v>
+        <v>130</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E63" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I63" s="2" t="s">
-        <v>49</v>
+        <v>135</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B64" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I64" s="4" t="s">
-        <v>50</v>
+      <c r="E64" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1436,112 +1505,112 @@
         <v>5</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>26</v>
+        <v>5</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D68" s="3" t="b">
+        <v>26</v>
+      </c>
+      <c r="I68" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D69" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I68" s="4" t="s">
+      <c r="I69" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I70" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I71" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I72" s="4" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I69" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I70" s="4" t="s">
+    <row r="73" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I73" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A71" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I71" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I72" s="4" t="s">
+    <row r="74" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A74" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I74" s="4" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A73" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I73" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A74" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I74" s="4" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1549,10 +1618,10 @@
         <v>5</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1560,21 +1629,21 @@
         <v>5</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1582,287 +1651,345 @@
         <v>5</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I78" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F79" s="3" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="I79" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F80" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="80" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A80" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="I80" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E84" s="3" t="b">
+        <v>44</v>
+      </c>
+      <c r="I84" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E85" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I84" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A85" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>46</v>
-      </c>
       <c r="I85" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="86" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I86" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I87" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A88" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="I88" s="7" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A87" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="I87" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A88" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E88" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I88" s="4" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="89" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
+      </c>
+      <c r="E89" s="3" t="b">
+        <v>1</v>
       </c>
       <c r="I89" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A90" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A91" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A92" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I92" s="4" t="s">
         <v>109</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A90" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I90" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A91" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I91" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A92" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I92" s="4" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="93" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="94" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I94" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A95" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I95" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A96" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="I96" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A97" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B97" s="3" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="95" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A95" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="I95" s="7" t="s">
+      <c r="C97" s="3" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="96" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A96" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B96" s="3" t="s">
+      <c r="D97" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I97" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D96" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A97" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I97" s="4" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="99" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A100" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="I100" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A101" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="E101" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I101" s="4" t="s">
-        <v>123</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A100" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I100" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A101" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="I101" s="7" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="102" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
+      </c>
+      <c r="E102" s="3" t="b">
+        <v>1</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="103" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I103" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A104" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I104" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A105" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I105" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A106" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I106" s="4" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A104" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I104" s="4" t="s">
+    <row r="107" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A107" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I107" s="4" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A108" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I108" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A109" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I109" s="4" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removes unused timeline-1 class from xlsx rows
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CAF856D-E9A1-5A4F-8140-C6B671534A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032D6DDE-6BD1-1442-BAF5-80A0F5F0CF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="139">
   <si>
     <t>class</t>
   </si>
@@ -53,9 +53,6 @@
     <t>content</t>
   </si>
   <si>
-    <t>timeline-1</t>
-  </si>
-  <si>
     <t>Before Nosgoth's Recorded History</t>
   </si>
   <si>
@@ -116,9 +113,6 @@
     <t>image</t>
   </si>
   <si>
-    <t>timeline-1 detail</t>
-  </si>
-  <si>
     <t>Millennia pass – at least 2,000 years</t>
   </si>
   <si>
@@ -281,9 +275,6 @@
     <t>Kain awakens in his mausoleum, and begins his "unlife" as a vampire.</t>
   </si>
   <si>
-    <t>timeline-1 game</t>
-  </si>
-  <si>
     <t>Kain finds his assassins and kills them, getting his revenge - but Mortanius drives him on to the Pillars, saying that the brigands were only the instruments of his murder, not the cause.</t>
   </si>
   <si>
@@ -308,18 +299,12 @@
     <t>#travel-1</t>
   </si>
   <si>
-    <t>timeline-1 time-travel travel-1</t>
-  </si>
-  <si>
     <t>BloodOmen</t>
   </si>
   <si>
     <t>Kain confronts William, each of them armed with the Soul Reaver (incarnations of the same weapon at different periods of time). Kain is victorious, and he triumphantly drinks the blood of the fallen king – this is witnessed by the king's guards, come to aid their martyred ruler.</t>
   </si>
   <si>
-    <t>timeline-1 time-travel paradox-1</t>
-  </si>
-  <si>
     <t>Kain discovers the Time Streaming Device and escapes back into the future – secure in his belief that he has thwarted Moebius's machinations by removing his pawn William from the game.</t>
   </si>
   <si>
@@ -350,9 +335,6 @@
     <t>Kain chooses the latter path, deciding to rule the world in its damnation rather than commit himself to oblivion. This apocalyptic act completes the Pillars' destruction – the Pillars topple as Kain seals their ruinous fate.</t>
   </si>
   <si>
-    <t>timeline-1 time-travel travel-1 detail</t>
-  </si>
-  <si>
     <t>Roughly 500 years after Blood Omen: Legacy of Kain</t>
   </si>
   <si>
@@ -389,9 +371,6 @@
     <t>Events of Legacy of Kain: Soul Reaver</t>
   </si>
   <si>
-    <t>timeline-1 time-travel travel-1 game</t>
-  </si>
-  <si>
     <t>Over the centuries, each of the vampires undergoes a series of evolutionary adaptations. These evolutionary "growth spurts" are preceded by a quiescent, near-hibernatory period of retreat, from which the vampire emerges transformed.</t>
   </si>
   <si>
@@ -440,16 +419,40 @@
     <t>SoulReaver2</t>
   </si>
   <si>
-    <t>timeline-1 time-travel travel-2 game</t>
-  </si>
-  <si>
-    <t>timeline-1 time-travel travel-2</t>
-  </si>
-  <si>
     <t>#SoulReaver2</t>
   </si>
   <si>
     <t>Raziel pursues Kain through Moebius's ancient Chronoplast time portal.</t>
+  </si>
+  <si>
+    <t>Raziel emerges from the Stronghold and sees past-Nosgoth for the first time.</t>
+  </si>
+  <si>
+    <t>Future Kain and Raziel both witness this event from the Pillars' clearing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> detail</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel travel-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel paradox-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel travel-2 game</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel travel-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> game</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel travel-1 detail</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel travel-1 game</t>
   </si>
 </sst>
 </file>
@@ -478,7 +481,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -488,6 +491,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -504,7 +525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -528,6 +549,24 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -864,7 +903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" style="3" customWidth="1"/>
@@ -879,16 +918,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -897,552 +936,417 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="D2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="3" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="E3" s="3" t="b">
         <v>1</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I4" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" s="4" t="s">
+    <row r="5" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I5" s="4" t="s">
+    <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="2" t="s">
+    <row r="7" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I7" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I7" s="4" t="s">
+    <row r="8" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I8" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I8" s="4" t="s">
+    <row r="9" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E9" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I10" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E9" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I10" s="4" t="s">
+    <row r="11" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I11" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="4" t="s">
+    <row r="12" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E12" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="2" t="s">
+    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="I13" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I13" s="4" t="s">
+    <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E14" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="2" t="s">
+    <row r="15" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I15" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I15" s="4" t="s">
+    <row r="16" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I16" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I16" s="5" t="s">
+    <row r="17" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I17" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I17" s="5" t="s">
+    <row r="18" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E18" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E18" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I18" s="2" t="s">
+    <row r="19" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I19" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I19" s="5" t="s">
+    <row r="20" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I20" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E21" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
     <row r="22" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I22" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I23" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>26</v>
+        <v>131</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="E25" s="3" t="b">
         <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I26" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I27" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
     <row r="28" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I28" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I29" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I30" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I29" s="5" t="s">
+    <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I31" s="4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I30" s="5" t="s">
+    <row r="32" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I32" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I31" s="4" t="s">
+    <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E33" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E33" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="I34" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>26</v>
+        <v>131</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I36" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I37" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I38" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I39" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E40" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I39" s="4" t="s">
+    <row r="41" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I41" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I42" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E40" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I40" s="2" t="s">
+    <row r="43" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I43" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I42" s="4" t="s">
+    <row r="44" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="I44" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I43" s="4" t="s">
+    <row r="45" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I45" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I44" s="4" t="s">
+    <row r="46" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I46" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A45" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I45" s="4" t="s">
+    <row r="47" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I47" s="4" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I46" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I47" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="48" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
-        <v>26</v>
+        <v>131</v>
       </c>
       <c r="I48" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I49" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
-        <v>5</v>
-      </c>
       <c r="I50" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E51" s="3" t="b">
         <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="G54" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A59" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B59" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D59" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I59" s="4" t="s">
-        <v>132</v>
+      <c r="B59" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D59" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I59" s="10" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1450,10 +1354,10 @@
         <v>135</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1461,10 +1365,10 @@
         <v>135</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" spans="1:9" ht="34" x14ac:dyDescent="0.2">
@@ -1472,10 +1376,10 @@
         <v>135</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1483,513 +1387,490 @@
         <v>135</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E64" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I64" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I64" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="E65" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B66" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I67" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B68" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I68" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I65" s="4" t="s">
+    <row r="69" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B69" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I69" s="4" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A66" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I66" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I67" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I68" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D69" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I69" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I70" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A71" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I71" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I72" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A73" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I73" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A74" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I74" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A75" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I75" s="4" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>44</v>
+        <v>131</v>
       </c>
       <c r="I76" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" s="11" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C77" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D77" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I77" s="12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B78" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B79" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I79" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B80" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I80" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B81" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I81" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B82" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I82" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B83" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I83" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B84" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I84" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B85" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I85" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B86" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I86" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="B87" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I87" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="B88" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I88" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A77" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I77" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A78" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I78" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I79" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A80" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I80" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A81" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C81" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="I81" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A82" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I82" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A83" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I83" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A84" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I84" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A85" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E85" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A86" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I86" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A87" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I87" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A88" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="I88" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E89" s="3" t="b">
-        <v>1</v>
+        <v>132</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>94</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="90" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E93" s="3" t="b">
+        <v>1</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="94" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
     </row>
     <row r="95" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
     </row>
     <row r="96" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A96" s="6" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
       <c r="I96" s="7" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
     </row>
     <row r="97" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D97" s="3" t="b">
+        <v>132</v>
+      </c>
+      <c r="E97" s="3" t="b">
         <v>1</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
     </row>
     <row r="99" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="I100" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A101" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A101" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I101" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="I101" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    </row>
+    <row r="102" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E102" s="3" t="b">
-        <v>1</v>
+        <v>132</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="I103" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A104" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I104" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A105" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I105" s="4" t="s">
-        <v>124</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A104" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="I104" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A105" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B105" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C105" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D105" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I105" s="14" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="106" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I106" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I107" s="4" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
     </row>
     <row r="108" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B108" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I108" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A109" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="I109" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A110" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E110" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I110" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="I108" s="4" t="s">
+    </row>
+    <row r="111" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A111" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I111" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A112" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I112" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A113" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I113" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A114" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I114" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A115" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I115" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A116" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I116" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A117" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F117" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="109" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A109" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B109" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F109" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="I109" s="4" t="s">
-        <v>137</v>
+      <c r="I117" s="4" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more modifications to functionality
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092BD0D7-8DDF-8B43-8A9B-8EB81B65D895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE9181E-8A8B-8E4B-9E8E-57C83DDCA097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="181">
   <si>
     <t>class</t>
   </si>
@@ -179,9 +179,6 @@
     <t>Human Raziel is born, and becomes a Sarafan warrior-priest</t>
   </si>
   <si>
-    <t>30 years pass</t>
-  </si>
-  <si>
     <t>Vorador crafts the Reaver blade, at the behest of Janos Audron. It is the most formidable weapon ever forged by the Vampires' swordsmiths – they infuse the blade with vampiric energy, empowering the Reaver to drain their enemies of their precious lifeblood.</t>
   </si>
   <si>
@@ -416,9 +413,6 @@
     <t>Raziel travels through Nosgoth, he discovers the Ancient Vampire temples and forges. Upon learning more about Nosgoth's history, he starts doubting the Elder God's power and intentions.</t>
   </si>
   <si>
-    <t>#paradox-2</t>
-  </si>
-  <si>
     <t>Raziel returns to the Sarafan fortress and encounters Kain before the tomb of William the Just.</t>
   </si>
   <si>
@@ -441,9 +435,6 @@
   </si>
   <si>
     <t>Stranded now in Nosgoth's nightmarish future, Raziel enters the ruined Pillars clearing for the first time, and sees the devastation wrought by Kain's fateful decision at the Pillars a century ago. In the gloom, Raziel meets the spectre of Ariel drifting restlessly among the toppled Pillars.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> time-travel paradox-2 detail</t>
   </si>
   <si>
     <t>Roughly 50 years after Blood Omen: Legacy of Kain</t>
@@ -566,6 +557,30 @@
   </si>
   <si>
     <t>enable</t>
+  </si>
+  <si>
+    <t>sr2-paradox-1</t>
+  </si>
+  <si>
+    <t>#sr2-paradox-1</t>
+  </si>
+  <si>
+    <t>30 years before Blood Omen: Legacy of Kain</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel sr2-paradox-1</t>
+  </si>
+  <si>
+    <t>30 years pass.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel SoulReaver2 sr2-paradox-1 undoneEvent</t>
+  </si>
+  <si>
+    <t>Raziel kills Kain with the Soul Reaver.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel sr2-paradox-1 detail</t>
   </si>
 </sst>
 </file>
@@ -1070,10 +1085,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.83203125" style="7" customWidth="1"/>
+    <col min="1" max="1" width="51.83203125" style="7" customWidth="1"/>
     <col min="2" max="2" width="23.33203125" style="7" customWidth="1"/>
     <col min="3" max="3" width="16" style="7" customWidth="1"/>
     <col min="4" max="5" width="10.83203125" style="7"/>
@@ -1107,7 +1122,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>24</v>
@@ -1229,7 +1244,7 @@
     </row>
     <row r="20" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="J20" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.2">
@@ -1242,17 +1257,17 @@
     </row>
     <row r="22" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J22" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="J23" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>25</v>
@@ -1263,42 +1278,42 @@
         <v>1</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J26" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J27" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="J28" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J29" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="J30" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J31" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="J32" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="17" x14ac:dyDescent="0.2">
@@ -1306,25 +1321,25 @@
         <v>1</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J34" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="J36" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="34" x14ac:dyDescent="0.2">
@@ -1352,38 +1367,38 @@
     </row>
     <row r="41" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="17" x14ac:dyDescent="0.2">
@@ -1393,57 +1408,57 @@
     </row>
     <row r="45" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J45" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="47" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="34" x14ac:dyDescent="0.2">
@@ -1453,49 +1468,49 @@
     </row>
     <row r="51" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="52" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="53" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="54" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>40</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="17" x14ac:dyDescent="0.2">
@@ -1525,7 +1540,7 @@
     </row>
     <row r="60" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J60" s="12" t="s">
         <v>36</v>
@@ -1533,206 +1548,206 @@
     </row>
     <row r="61" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J61" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J62" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="63" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B63" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E63" s="19" t="b">
         <v>1</v>
       </c>
       <c r="J63" s="21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="64" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B64" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J64" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B65" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J65" s="20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B66" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="G66" s="19" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="J66" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="67" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="19" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B67" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J67" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="68" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" s="19" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B68" s="19" t="s">
         <v>39</v>
       </c>
       <c r="F68" s="19" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H68" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J68" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="69" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A69" s="19" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B69" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J69" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="70" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="19" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B70" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J70" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="71" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D71" s="3" t="b">
         <v>1</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A72" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J72" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A72" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J72" s="12" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="73" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J73" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="74" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J75" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="76" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J76" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="E77" s="7" t="b">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="E78" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="J77" s="6" t="s">
+      <c r="J78" s="6" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B78" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J78" s="20" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="79" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1740,139 +1755,142 @@
         <v>39</v>
       </c>
       <c r="J79" s="20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B80" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J80" s="20" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B80" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J80" s="20" t="s">
+    <row r="81" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B81" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J81" s="20" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="81" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A81" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J81" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J83" s="2" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
     </row>
     <row r="84" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J84" s="2" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
     </row>
     <row r="85" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G85" s="1" t="s">
-        <v>126</v>
-      </c>
       <c r="J85" s="2" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
     </row>
     <row r="86" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F86" s="1" t="s">
-        <v>153</v>
+      <c r="G86" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="J86" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A87" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J87" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A87" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="J87" s="8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="J88" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A90" s="7" t="s">
+    <row r="89" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A92" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J92" s="12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A93" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="J90" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A91" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="B91" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C91" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="D91" s="13" t="b">
+      <c r="B93" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C93" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D93" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="J91" s="14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B92" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J92" s="20" t="s">
+      <c r="J93" s="14" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B93" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J93" s="20" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="94" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1880,7 +1898,7 @@
         <v>39</v>
       </c>
       <c r="J94" s="20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="95" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1888,7 +1906,7 @@
         <v>39</v>
       </c>
       <c r="J95" s="20" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="96" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1896,7 +1914,7 @@
         <v>39</v>
       </c>
       <c r="J96" s="20" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="97" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1904,15 +1922,15 @@
         <v>39</v>
       </c>
       <c r="J97" s="20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="B98" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J98" s="20" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="99" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1920,7 +1938,7 @@
         <v>39</v>
       </c>
       <c r="J99" s="20" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="100" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1928,430 +1946,446 @@
         <v>39</v>
       </c>
       <c r="J100" s="20" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B101" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J101" s="20" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="102" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B102" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F102" s="19" t="s">
-        <v>145</v>
-      </c>
       <c r="J102" s="20" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="103" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A103" s="19" t="s">
-        <v>143</v>
-      </c>
       <c r="B103" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C103" s="19" t="s">
-        <v>149</v>
-      </c>
       <c r="J103" s="20" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="104" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A104" s="19" t="s">
-        <v>143</v>
-      </c>
       <c r="B104" s="19" t="s">
         <v>39</v>
       </c>
+      <c r="F104" s="19" t="s">
+        <v>142</v>
+      </c>
       <c r="J104" s="20" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A105" s="19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B105" s="19" t="s">
         <v>39</v>
       </c>
+      <c r="C105" s="19" t="s">
+        <v>146</v>
+      </c>
       <c r="J105" s="20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A106" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="B106" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J106" s="20" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A106" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="B106" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J106" s="20" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="107" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A107" s="19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B107" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E107" s="19" t="b">
+      <c r="J107" s="20" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A108" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="B108" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J108" s="20" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A109" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="B109" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E109" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="J107" s="20" t="s">
+      <c r="J109" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A110" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J110" s="20" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="108" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A108" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="B108" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J108" s="20" t="s">
+    <row r="111" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A111" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J111" s="20" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="109" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A109" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="B109" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J109" s="20" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A110" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="J110" s="12" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A111" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B111" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J111" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A112" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B112" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J112" s="2" t="s">
-        <v>132</v>
+    <row r="112" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A112" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="J112" s="12" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="113" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="C113" s="1" t="s">
+        <v>155</v>
+      </c>
       <c r="J113" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J114" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J115" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="116" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J116" s="2" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
     </row>
     <row r="117" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F117" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="J117" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A118" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="J118" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A120" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="J120" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A121" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E121" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J121" s="8" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A119" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="E119" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J119" s="8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A120" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="J120" s="8" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A121" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="J121" s="8" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A122" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="J122" s="8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A123" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="J123" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A124" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="J124" s="8" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A125" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J125" s="8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A126" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J126" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A127" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J127" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A128" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="J125" s="8" t="s">
+      <c r="J128" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A126" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="J126" s="12" t="s">
+    <row r="129" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A129" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="B129" s="15" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="127" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A127" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="B127" s="15" t="s">
+      <c r="C129" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="C127" s="15" t="s">
+      <c r="D129" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J129" s="16" t="s">
         <v>103</v>
-      </c>
-      <c r="D127" s="15" t="b">
-        <v>1</v>
-      </c>
-      <c r="J127" s="16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A128" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="B128" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="J128" s="18" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A129" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="B129" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="J129" s="18" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="130" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A130" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B130" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J130" s="18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A131" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B131" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J131" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A132" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B132" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J132" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A133" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="B130" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="J130" s="18" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A131" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="J131" s="12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A132" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="B132" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="E132" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="J132" s="18" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A133" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="B133" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="J133" s="18" t="s">
-        <v>108</v>
+      <c r="J133" s="12" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="134" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A134" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B134" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="E134" s="17" t="b">
+        <v>1</v>
       </c>
       <c r="J134" s="18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A135" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B135" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J135" s="18" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A136" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B136" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J136" s="18" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="137" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A137" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B137" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J137" s="18" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="138" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A138" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B138" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J138" s="18" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A139" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B139" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="F139" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J139" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A140" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B140" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J140" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A141" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B141" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F141" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="H141" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="J141" s="18" t="s">
         <v>120</v>
-      </c>
-      <c r="H139" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="J139" s="18" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
further work on timeline, adds defiance and bo2 entries
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE9181E-8A8B-8E4B-9E8E-57C83DDCA097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{919F6050-795F-3548-ABFD-E5A2B8398CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
+    <workbookView xWindow="-20" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
   <sheets>
     <sheet name="timeline" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="191">
   <si>
     <t>class</t>
   </si>
@@ -419,9 +419,6 @@
     <t xml:space="preserve">Elder Kain, by unknown means, also travels to Nosgoth's future. </t>
   </si>
   <si>
-    <t xml:space="preserve"> time-travel paradox-2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Raziel pressures Moebius into using the Chronoplast chamber to send him to Nosgoth's past - so he can learn more about the Ancient Vampires and his own role in history. </t>
   </si>
   <si>
@@ -447,9 +444,6 @@
   </si>
   <si>
     <t>Raziel enters the ruined village of Uschtenheim for the first time.</t>
-  </si>
-  <si>
-    <t>Raziel enters the canyon, and meets Soul Reaver-era Kain at the ruins of Janos Audron's Retreat – in this era, the majestic facades of the Vampires' ancient cliff-dwellings are collapsed and toppled.</t>
   </si>
   <si>
     <t>After enhancing the Reaver with the Elemental power of Air, Raziel accesses and activates the time-streaming device in the Swamp.</t>
@@ -553,9 +547,6 @@
 Kain intervenes, stopping the blade from consuming Raziel's soul. In doing so, he creates another time paradox. Raziel, nearly destroyed by the Reaver, comes to a grim realization—his terrible destiny is inescapable, and Kain has only delayed the inevitable.</t>
   </si>
   <si>
-    <t>#paradox-3</t>
-  </si>
-  <si>
     <t>enable</t>
   </si>
   <si>
@@ -581,6 +572,45 @@
   </si>
   <si>
     <t xml:space="preserve"> time-travel sr2-paradox-1 detail</t>
+  </si>
+  <si>
+    <t>Raziel enters the canyon, and meets the Elder Kain at the ruins of Janos Audron's Retreat – in this era, the majestic facades of the Vampires' ancient cliff-dwellings are collapsed and toppled.</t>
+  </si>
+  <si>
+    <t>bo.png</t>
+  </si>
+  <si>
+    <t>sr.png</t>
+  </si>
+  <si>
+    <t>sr2.png</t>
+  </si>
+  <si>
+    <t>500 years before Blood Omen: Legacy of Kain</t>
+  </si>
+  <si>
+    <t>#sr2-paradox-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel SoulReaver2 sr2-paradox-2 undoneEvent</t>
+  </si>
+  <si>
+    <t>Wraith Raziel is consumend by the  Reaver blade, becoming the soul Devouring entity trapped within it.</t>
+  </si>
+  <si>
+    <t>The Soul Reaver sword is found beside the dead body of Sarafan Raziel. The blade is taken to Avernus Cathedral.</t>
+  </si>
+  <si>
+    <t>Elder Kain takes the Blood Reaver blade with him as his weapon - he set's out to find Moebius to gain clarity on Raziel's whereabouts</t>
+  </si>
+  <si>
+    <t>Raziel, weakened by almost being absorved by the blade - fades into the Spectral Realm - away from Kain's reach.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel sr2-paradox-2</t>
+  </si>
+  <si>
+    <t>BO2,DEF</t>
   </si>
 </sst>
 </file>
@@ -1085,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.83203125" style="7" customWidth="1"/>
@@ -1122,7 +1152,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>24</v>
@@ -1365,61 +1395,58 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>139</v>
+    <row r="41" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J41" s="11" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="42" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="C42" s="1" t="s">
+        <v>150</v>
+      </c>
       <c r="J42" s="2" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J44" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J45" s="8" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>40</v>
@@ -1430,515 +1457,533 @@
     </row>
     <row r="47" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J48" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B47" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="J50" s="8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="J51" s="8" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="52" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J55" s="8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J54" s="8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A56" s="7" t="s">
+        <v>184</v>
+      </c>
       <c r="J56" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A57" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="J57" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="J61" s="8" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J57" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J58" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J59" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A60" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="J60" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J61" s="8" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J62" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J63" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J64" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A65" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J65" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J66" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J67" s="8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="63" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A63" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B63" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="E63" s="19" t="b">
+    <row r="68" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A68" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B68" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C68" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="E68" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="J63" s="21" t="s">
+      <c r="J68" s="21" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A64" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B64" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J64" s="20" t="s">
+    <row r="69" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A69" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B69" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J69" s="20" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A65" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B65" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J65" s="20" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A66" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B66" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C66" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="G66" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="J66" s="20" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A67" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="B67" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J67" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A68" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="B68" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F68" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="H68" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="J68" s="20" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A69" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="B69" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J69" s="20" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="70" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="19" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="B70" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J70" s="20" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A71" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B71" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="G71" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="J71" s="20" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A72" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B72" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J72" s="20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A73" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B73" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F73" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="H73" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="J73" s="20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A74" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B74" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J74" s="20" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A75" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B75" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J75" s="20" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A71" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C71" s="3" t="s">
+    <row r="76" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D71" s="3" t="b">
+      <c r="D76" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="J71" s="4" t="s">
+      <c r="I76" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="J76" s="4" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="72" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A72" s="10" t="s">
+    <row r="77" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="J72" s="12" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A73" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J73" s="2" t="s">
+      <c r="J77" s="12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J78" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="74" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A74" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J74" s="2" t="s">
+    <row r="79" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J79" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A75" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J75" s="2" t="s">
+    <row r="80" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J80" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A76" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J76" s="2" t="s">
+    <row r="81" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J81" s="2" t="s">
         <v>116</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A77" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J77" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="E78" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J78" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B79" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J79" s="20" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B80" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J80" s="20" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B81" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J81" s="20" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="82" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A83" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J83" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="E83" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B84" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J84" s="20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B85" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J85" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B86" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J86" s="20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J88" s="2" t="s">
         <v>124</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A84" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J84" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A85" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J85" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A86" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G86" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="J86" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A87" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="J87" s="8" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A88" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="J88" s="2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="89" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A92" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="J92" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C89" s="1" t="s">
+    </row>
+    <row r="93" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J89" s="2" t="s">
+      <c r="B94" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J94" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="92" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A92" s="10" t="s">
+    <row r="97" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A97" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="J92" s="12" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A93" s="13" t="s">
+      <c r="J97" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A98" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="B93" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C93" s="13" t="s">
+      <c r="B98" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C98" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="D93" s="13" t="b">
+      <c r="D98" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="J93" s="14" t="s">
+      <c r="I98" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="J98" s="14" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="94" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B94" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J94" s="20" t="s">
+    <row r="99" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B99" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J99" s="20" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B95" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J95" s="20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B96" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J96" s="20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B97" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J97" s="20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B98" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J98" s="20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B99" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J99" s="20" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="100" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1946,15 +1991,15 @@
         <v>39</v>
       </c>
       <c r="J100" s="20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="B101" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J101" s="20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="102" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1962,7 +2007,7 @@
         <v>39</v>
       </c>
       <c r="J102" s="20" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="103" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1970,421 +2015,464 @@
         <v>39</v>
       </c>
       <c r="J103" s="20" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="104" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B104" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F104" s="19" t="s">
-        <v>142</v>
-      </c>
       <c r="J104" s="20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B105" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J105" s="20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B106" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J106" s="20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B107" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J107" s="20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B108" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J108" s="20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B109" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F109" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="J109" s="20" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A105" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B105" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C105" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="J105" s="20" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A106" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B106" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J106" s="20" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A107" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B107" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J107" s="20" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A108" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B108" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J108" s="20" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A109" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B109" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E109" s="19" t="b">
-        <v>1</v>
-      </c>
-      <c r="J109" s="20" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="110" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A110" s="19" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B110" s="19" t="s">
         <v>39</v>
       </c>
+      <c r="C110" s="19" t="s">
+        <v>144</v>
+      </c>
       <c r="J110" s="20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A111" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B111" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J111" s="20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A112" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B112" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J112" s="20" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A113" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B113" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J113" s="20" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A114" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B114" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E114" s="19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J114" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A115" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B115" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J115" s="20" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="111" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A111" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B111" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J111" s="20" t="s">
+    <row r="116" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A116" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B116" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J116" s="20" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="112" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A112" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J112" s="12" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A113" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B113" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="J113" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A114" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B114" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J114" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A115" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B115" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J115" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A116" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B116" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J116" s="2" t="s">
+    <row r="117" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A117" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="J117" s="12" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A117" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B117" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J117" s="2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="118" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="C118" s="1" t="s">
+        <v>153</v>
+      </c>
       <c r="J118" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
     </row>
     <row r="119" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J120" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A121" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J121" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J122" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F124" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B119" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F119" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="J119" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A120" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="J120" s="12" t="s">
+      <c r="J124" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A125" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="J125" s="12" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A121" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="E121" s="7" t="b">
+    <row r="126" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A126" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E126" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="J121" s="8" t="s">
+      <c r="J126" s="8" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A122" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="J122" s="8" t="s">
+    <row r="127" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A127" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J127" s="8" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A123" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="J123" s="8" t="s">
+    <row r="128" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A128" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J128" s="8" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A124" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="J124" s="8" t="s">
+    <row r="129" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A129" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J129" s="8" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A125" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="J125" s="8" t="s">
+    <row r="130" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A130" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J130" s="8" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A126" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="J126" s="8" t="s">
+    <row r="131" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A131" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J131" s="8" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A127" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="J127" s="8" t="s">
+    <row r="132" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A132" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J132" s="8" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A128" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="J128" s="12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A129" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="B129" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="C129" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="D129" s="15" t="b">
-        <v>1</v>
-      </c>
-      <c r="J129" s="16" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A130" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="B130" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J130" s="18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A131" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="B131" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J131" s="18" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A132" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="B132" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J132" s="18" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="133" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A133" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J133" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="134" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A134" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="B134" s="17" t="s">
+    <row r="134" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A134" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="B134" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="E134" s="17" t="b">
+      <c r="C134" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="D134" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="J134" s="18" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="I134" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="J134" s="16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A135" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B135" s="17" t="s">
         <v>101</v>
       </c>
       <c r="J135" s="18" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="136" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A136" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B136" s="17" t="s">
         <v>101</v>
       </c>
       <c r="J136" s="18" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="137" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A137" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B137" s="17" t="s">
         <v>101</v>
       </c>
       <c r="J137" s="18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A138" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="B138" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J138" s="18" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A138" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="J138" s="12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A139" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B139" s="17" t="s">
         <v>101</v>
       </c>
+      <c r="E139" s="17" t="b">
+        <v>1</v>
+      </c>
       <c r="J139" s="18" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A140" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B140" s="17" t="s">
         <v>101</v>
       </c>
       <c r="J140" s="18" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="141" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A141" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B141" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F141" s="17" t="s">
+      <c r="J141" s="18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A142" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B142" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J142" s="18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A143" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B143" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J143" s="18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A144" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B144" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J144" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A145" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B145" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J145" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A146" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B146" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F146" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="H141" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="J141" s="18" t="s">
+      <c r="H146" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="J146" s="18" t="s">
         <v>120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
udpates timeline, updates paradox and time travel event cards
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{919F6050-795F-3548-ABFD-E5A2B8398CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0F1DAA-2806-3447-BAAF-D402A4516808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
   <sheets>
     <sheet name="timeline" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="207">
   <si>
     <t>class</t>
   </si>
@@ -601,16 +601,64 @@
     <t>The Soul Reaver sword is found beside the dead body of Sarafan Raziel. The blade is taken to Avernus Cathedral.</t>
   </si>
   <si>
-    <t>Elder Kain takes the Blood Reaver blade with him as his weapon - he set's out to find Moebius to gain clarity on Raziel's whereabouts</t>
-  </si>
-  <si>
-    <t>Raziel, weakened by almost being absorved by the blade - fades into the Spectral Realm - away from Kain's reach.</t>
+    <t>DEF</t>
   </si>
   <si>
     <t xml:space="preserve"> time-travel sr2-paradox-2</t>
   </si>
   <si>
     <t>BO2,DEF</t>
+  </si>
+  <si>
+    <t>Raziel, weakened by almost being absorved by the blade, fades into the Spectral Realm - away from Kain's reach.</t>
+  </si>
+  <si>
+    <t>Defiance</t>
+  </si>
+  <si>
+    <t>defiance.png</t>
+  </si>
+  <si>
+    <t>Events of Legacy of Kain: Defiance</t>
+  </si>
+  <si>
+    <t>Kain spends years searching , after failing to succeed - he returns to the Sarafan Keep to question Moebius on Raziel's whereabouts.</t>
+  </si>
+  <si>
+    <t>Elder Kain takes the Blood Reaver blade with him as his weapon - he set's out tofind Raziel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel sr2-paradox-2 defiance game</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel sr2-paradox-2 defiance</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time-travel sr2-paradox-2 detail</t>
+  </si>
+  <si>
+    <t>Years pass.</t>
+  </si>
+  <si>
+    <t>Kain finds Moebius in the depths of an underground cavern in the Keep. The Time Streamer is seen seemingly speaking to an unknown entity.</t>
+  </si>
+  <si>
+    <t>Moebius activates his staff, weakining Kain with it's sorcery. Then proceeds to taunt Kain, placing blame on him for an 'unleashed' Raziel.</t>
+  </si>
+  <si>
+    <t>Wraith Raziel remains in the Elder God's lair within the Underworld.  Time stands still in the Spectral Realm, meaning he has spent nearly 500 years since almost being absorbed by the Reaver blade.</t>
+  </si>
+  <si>
+    <t>After trying to feign submission to the Elder God, Raziel narrowly escapes the Underworld. The Elder God is enraged by Raziel's actions.</t>
+  </si>
+  <si>
+    <t>Raziel emerges emerges from the Underworld at a Cementery, discovering the place was also human Kain's resting place.</t>
+  </si>
+  <si>
+    <t>Raziel finds portals to the Ancient Vampire Citadel, where he forges the Spectral Reaver with the Elemental powers of Light and Dark.</t>
+  </si>
+  <si>
+    <t>Raziel sets out to complete the task he couldn't finish 500 years ago; finding Janos Audron to discover more about his own purpose.</t>
   </si>
 </sst>
 </file>
@@ -639,7 +687,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -688,6 +736,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF5400"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFC854D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -716,7 +782,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -781,12 +847,37 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFC854D"/>
+      <color rgb="FFFF5400"/>
+      <color rgb="FFCE3100"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1115,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.83203125" style="7" customWidth="1"/>
@@ -1124,7 +1215,7 @@
     <col min="4" max="5" width="10.83203125" style="7"/>
     <col min="6" max="6" width="14" style="7" customWidth="1"/>
     <col min="7" max="8" width="14.33203125" style="7" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" style="7"/>
+    <col min="9" max="9" width="14.83203125" style="7" customWidth="1"/>
     <col min="10" max="10" width="145.83203125" style="8" customWidth="1"/>
     <col min="11" max="16384" width="10.83203125" style="7"/>
   </cols>
@@ -1569,7 +1660,7 @@
         <v>183</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J58" s="2" t="s">
         <v>168</v>
@@ -1577,283 +1668,295 @@
     </row>
     <row r="59" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J59" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" s="26" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A60" s="26" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A60" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J60" s="2" t="s">
+      <c r="J60" s="27" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A61" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="J61" s="12" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" s="26" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A62" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="J62" s="27" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" s="22" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A63" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B63" s="22" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="J61" s="8" t="s">
+      <c r="C63" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="D63" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I63" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="J63" s="23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A64" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B64" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J64" s="25" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A65" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B65" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J65" s="25" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="J66" s="8" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J62" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J63" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J64" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A65" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="J65" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J66" s="8" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J67" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J68" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J69" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A70" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J70" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J71" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J72" s="8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="68" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A68" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B68" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C68" s="19" t="s">
+    <row r="73" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A73" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B73" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C73" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E68" s="19" t="b">
+      <c r="E73" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="J68" s="21" t="s">
+      <c r="J73" s="21" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="69" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A69" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B69" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J69" s="20" t="s">
+    <row r="74" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A74" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B74" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J74" s="20" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A70" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B70" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J70" s="20" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A71" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B71" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C71" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="G71" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="J71" s="20" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A72" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="B72" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J72" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A73" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="B73" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F73" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="H73" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="J73" s="20" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A74" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="B74" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J74" s="20" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="75" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B75" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J75" s="20" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A76" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B76" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C76" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="G76" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="J76" s="20" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B75" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J75" s="20" t="s">
+      <c r="B77" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J77" s="20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A78" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B78" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F78" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="H78" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="J78" s="20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A79" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B79" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J79" s="20" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A80" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B80" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J80" s="20" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A76" s="3" t="s">
+    <row r="81" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B76" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C76" s="3" t="s">
+      <c r="B81" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C81" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D76" s="3" t="b">
+      <c r="D81" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I76" s="3" t="s">
+      <c r="I81" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="J76" s="4" t="s">
+      <c r="J81" s="4" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A77" s="10" t="s">
+    <row r="82" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A82" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="J77" s="12" t="s">
+      <c r="J82" s="12" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="78" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A78" s="1" t="s">
+    <row r="83" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B78" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J78" s="2" t="s">
+      <c r="B83" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J83" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A79" s="1" t="s">
+    <row r="84" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J79" s="2" t="s">
+      <c r="B84" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J84" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A80" s="1" t="s">
+    <row r="85" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J80" s="2" t="s">
+      <c r="B85" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J85" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="81" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A81" s="1" t="s">
+    <row r="86" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B81" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J81" s="2" t="s">
+      <c r="B86" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J86" s="2" t="s">
         <v>116</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A82" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J82" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="E83" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B84" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J84" s="20" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B85" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J85" s="20" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B86" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J86" s="20" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="87" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -1864,166 +1967,169 @@
         <v>40</v>
       </c>
       <c r="J87" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="E88" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B89" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J89" s="20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B90" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J90" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B91" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J91" s="20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J92" s="2" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="88" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A88" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J88" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A89" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J89" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A90" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J90" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A91" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G91" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J91" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A92" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="J92" s="8" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C93" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F93" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="J93" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="94" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J95" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A97" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="J97" s="8" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B94" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J94" s="2" t="s">
+      <c r="B99" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J99" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A97" s="10" t="s">
+    <row r="102" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A102" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="J97" s="12" t="s">
+      <c r="J102" s="12" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A98" s="13" t="s">
+    <row r="103" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A103" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="B98" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C98" s="13" t="s">
+      <c r="B103" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C103" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="D98" s="13" t="b">
+      <c r="D103" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="I98" s="19" t="s">
+      <c r="I103" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="J98" s="14" t="s">
+      <c r="J103" s="14" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="99" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B99" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J99" s="20" t="s">
+    <row r="104" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B104" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J104" s="20" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B100" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J100" s="20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B101" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J101" s="20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B102" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J102" s="20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B103" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J103" s="20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B104" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J104" s="20" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="105" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2031,15 +2137,15 @@
         <v>39</v>
       </c>
       <c r="J105" s="20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="B106" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J106" s="20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="107" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2047,7 +2153,7 @@
         <v>39</v>
       </c>
       <c r="J107" s="20" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="108" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -2055,79 +2161,58 @@
         <v>39</v>
       </c>
       <c r="J108" s="20" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="109" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B109" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F109" s="19" t="s">
+      <c r="J109" s="20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B110" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J110" s="20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B111" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J111" s="20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B112" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J112" s="20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B113" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J113" s="20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B114" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F114" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="J109" s="20" t="s">
+      <c r="J114" s="20" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A110" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B110" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C110" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="J110" s="20" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A111" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B111" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J111" s="20" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A112" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B112" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J112" s="20" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A113" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B113" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J113" s="20" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A114" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B114" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E114" s="19" t="b">
-        <v>1</v>
-      </c>
-      <c r="J114" s="20" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="115" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -2137,315 +2222,321 @@
       <c r="B115" s="19" t="s">
         <v>39</v>
       </c>
+      <c r="C115" s="19" t="s">
+        <v>144</v>
+      </c>
       <c r="J115" s="20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A116" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B116" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J116" s="20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A117" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B117" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J117" s="20" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A118" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B118" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J118" s="20" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" s="24" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A119" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B119" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J119" s="25" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A120" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B120" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J120" s="25" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A121" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B121" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J121" s="25" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A122" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B122" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J122" s="25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A123" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B123" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J123" s="25" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A124" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B124" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E124" s="19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J124" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A125" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B125" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J125" s="20" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="116" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A116" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B116" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J116" s="20" t="s">
+    <row r="126" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A126" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B126" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J126" s="20" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="117" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A117" s="10" t="s">
+    <row r="127" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A127" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="J117" s="12" t="s">
+      <c r="J127" s="12" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="118" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A118" s="1" t="s">
+    <row r="128" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A128" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B118" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C118" s="1" t="s">
+      <c r="B128" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C128" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="J118" s="2" t="s">
+      <c r="J128" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="119" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A119" s="1" t="s">
+    <row r="129" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A129" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B119" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J119" s="2" t="s">
+      <c r="B129" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J129" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="120" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A120" s="1" t="s">
+    <row r="130" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B120" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J120" s="2" t="s">
+      <c r="B130" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J130" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="121" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A121" s="1" t="s">
+    <row r="131" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B121" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J121" s="2" t="s">
+      <c r="B131" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J131" s="2" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="122" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A122" s="1" t="s">
+    <row r="132" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A132" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B122" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J122" s="2" t="s">
+      <c r="B132" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J132" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="123" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A123" s="1" t="s">
+    <row r="133" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A133" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B123" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J123" s="2" t="s">
+      <c r="B133" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J133" s="2" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="124" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A124" s="1" t="s">
+    <row r="134" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A134" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B124" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F124" s="1" t="s">
+      <c r="B134" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F134" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="J124" s="2" t="s">
+      <c r="J134" s="2" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="125" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A125" s="10" t="s">
+    <row r="135" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A135" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="J125" s="12" t="s">
+      <c r="J135" s="12" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A126" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="E126" s="7" t="b">
+    <row r="136" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A136" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E136" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="J126" s="8" t="s">
+      <c r="J136" s="8" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A127" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J127" s="8" t="s">
+    <row r="137" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A137" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J137" s="8" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A128" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J128" s="8" t="s">
+    <row r="138" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A138" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J138" s="8" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A129" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J129" s="8" t="s">
+    <row r="139" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A139" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J139" s="8" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="130" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A130" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J130" s="8" t="s">
+    <row r="140" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A140" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J140" s="8" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A131" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J131" s="8" t="s">
+    <row r="141" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A141" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J141" s="8" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A132" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J132" s="8" t="s">
+    <row r="142" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A142" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J142" s="8" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="133" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A133" s="10" t="s">
+    <row r="143" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A143" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="J133" s="12" t="s">
+      <c r="J143" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="134" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A134" s="15" t="s">
+    <row r="144" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A144" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="B134" s="15" t="s">
+      <c r="B144" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="C134" s="15" t="s">
+      <c r="C144" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="D134" s="15" t="b">
+      <c r="D144" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="I134" s="15" t="s">
+      <c r="I144" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="J134" s="16" t="s">
+      <c r="J144" s="16" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A135" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B135" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J135" s="18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A136" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B136" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J136" s="18" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A137" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B137" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J137" s="18" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A138" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="J138" s="12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A139" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B139" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="E139" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="J139" s="18" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A140" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B140" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J140" s="18" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A141" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B141" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J141" s="18" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A142" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B142" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J142" s="18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A143" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B143" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J143" s="18" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A144" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B144" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J144" s="18" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="145" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -2456,7 +2547,7 @@
         <v>101</v>
       </c>
       <c r="J145" s="18" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="146" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2466,13 +2557,123 @@
       <c r="B146" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F146" s="17" t="s">
+      <c r="J146" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A147" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B147" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J147" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A148" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="J148" s="12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A149" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B149" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="E149" s="17" t="b">
+        <v>1</v>
+      </c>
+      <c r="J149" s="18" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A150" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B150" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J150" s="18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A151" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B151" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J151" s="18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A152" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B152" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J152" s="18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A153" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B153" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J153" s="18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A154" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B154" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J154" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A155" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B155" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J155" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A156" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B156" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F156" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="H146" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="J146" s="18" t="s">
+      <c r="H156" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="J156" s="18" t="s">
         <v>120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
more improvements to funcitonality and content
</commit_message>
<xml_diff>
--- a/public/content/timeline.xlsx
+++ b/public/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/public/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0F1DAA-2806-3447-BAAF-D402A4516808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073ACFAD-FFEA-A847-9886-D8E1F777A5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="207">
   <si>
     <t>class</t>
   </si>
@@ -1206,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J160"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.83203125" style="7" customWidth="1"/>
@@ -1743,223 +1743,223 @@
         <v>201</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="J66" s="8" t="s">
+    <row r="66" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A66" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B66" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J66" s="25" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A67" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B67" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J67" s="25" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A68" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B68" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J68" s="25" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A69" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B69" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J69" s="25" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="J70" s="8" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J67" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J68" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="J69" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A70" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="J70" s="12" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J71" s="8" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="J72" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J73" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A74" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J74" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J75" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="J76" s="8" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A73" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B73" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C73" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E73" s="19" t="b">
-        <v>1</v>
-      </c>
-      <c r="J73" s="21" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A74" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B74" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J74" s="20" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A75" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B75" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J75" s="20" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A76" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B76" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C76" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="G76" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="J76" s="20" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="77" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B77" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C77" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="E77" s="19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J77" s="21" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A78" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B78" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J78" s="20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B79" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J79" s="20" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A80" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B80" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C80" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="G80" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="J80" s="20" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B77" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J77" s="20" t="s">
+      <c r="B81" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J81" s="20" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="78" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A78" s="19" t="s">
+    <row r="82" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A82" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B78" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F78" s="19" t="s">
+      <c r="B82" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F82" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="H78" s="19" t="s">
+      <c r="H82" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="J78" s="20" t="s">
+      <c r="J82" s="20" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A79" s="19" t="s">
+    <row r="83" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A83" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B79" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J79" s="20" t="s">
+      <c r="B83" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J83" s="20" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A80" s="19" t="s">
+    <row r="84" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A84" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B80" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J80" s="20" t="s">
+      <c r="B84" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J84" s="20" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="81" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A81" s="3" t="s">
+    <row r="85" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A85" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="J85" s="12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B81" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C81" s="3" t="s">
+      <c r="B86" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C86" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D81" s="3" t="b">
+      <c r="D86" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I81" s="3" t="s">
+      <c r="I86" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="J81" s="4" t="s">
+      <c r="J86" s="4" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="82" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A82" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="J82" s="12" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A83" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J83" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A84" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J84" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A85" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J85" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A86" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J86" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>152</v>
       </c>
@@ -1967,83 +1967,83 @@
         <v>40</v>
       </c>
       <c r="J87" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J91" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="E88" s="7" t="b">
+    <row r="92" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="E92" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="J88" s="6" t="s">
+      <c r="J92" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="89" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B89" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J89" s="20" t="s">
+    <row r="93" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B93" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J93" s="20" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="90" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B90" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J90" s="20" t="s">
+    <row r="94" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B94" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J94" s="20" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="91" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B91" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J91" s="20" t="s">
+    <row r="95" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B95" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J95" s="20" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A92" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J92" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A93" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J93" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A94" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J94" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A95" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J95" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="96" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2053,19 +2053,19 @@
       <c r="B96" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G96" s="1" t="s">
-        <v>171</v>
-      </c>
       <c r="J96" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A97" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="J97" s="8" t="s">
-        <v>176</v>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="98" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2075,85 +2075,97 @@
       <c r="B98" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C98" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F98" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="J98" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="99" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A100" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="J100" s="8" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B99" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J99" s="2" t="s">
+      <c r="B103" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J103" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="102" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A102" s="10" t="s">
+    <row r="106" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A106" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="J102" s="12" t="s">
+      <c r="J106" s="12" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="103" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A103" s="13" t="s">
+    <row r="107" spans="1:10" s="13" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A107" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="B103" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C103" s="13" t="s">
+      <c r="B107" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C107" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="D103" s="13" t="b">
+      <c r="D107" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="I103" s="19" t="s">
+      <c r="I107" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="J103" s="14" t="s">
+      <c r="J107" s="14" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B104" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J104" s="20" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B105" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J105" s="20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B106" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J106" s="20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B107" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J107" s="20" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="108" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -2161,7 +2173,7 @@
         <v>39</v>
       </c>
       <c r="J108" s="20" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="109" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2169,15 +2181,15 @@
         <v>39</v>
       </c>
       <c r="J109" s="20" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="B110" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J110" s="20" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="111" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2185,128 +2197,116 @@
         <v>39</v>
       </c>
       <c r="J111" s="20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="B112" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J112" s="20" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B113" s="19" t="s">
         <v>39</v>
       </c>
       <c r="J113" s="20" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="114" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B114" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F114" s="19" t="s">
+      <c r="J114" s="20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B115" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J115" s="20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B116" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J116" s="20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B117" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J117" s="20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B118" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F118" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="J114" s="20" t="s">
+      <c r="J118" s="20" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="115" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A115" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B115" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C115" s="19" t="s">
+    <row r="119" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A119" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B119" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C119" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="J115" s="20" t="s">
+      <c r="J119" s="20" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="116" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A116" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B116" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J116" s="20" t="s">
+    <row r="120" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A120" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B120" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J120" s="20" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="117" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A117" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B117" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J117" s="20" t="s">
+    <row r="121" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A121" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B121" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J121" s="20" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="118" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A118" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B118" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J118" s="20" t="s">
+    <row r="122" spans="1:10" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A122" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B122" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J122" s="20" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="119" spans="1:10" s="24" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A119" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="B119" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="J119" s="25" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A120" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="B120" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="J120" s="25" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A121" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="B121" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="J121" s="25" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A122" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="B122" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="J122" s="25" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10" s="24" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A123" s="24" t="s">
         <v>197</v>
       </c>
@@ -2314,112 +2314,112 @@
         <v>187</v>
       </c>
       <c r="J123" s="25" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A124" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B124" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J124" s="25" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A125" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B125" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J125" s="25" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A126" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B126" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J126" s="25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" s="24" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A127" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B127" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="J127" s="25" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="124" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A124" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B124" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E124" s="19" t="b">
+    <row r="128" spans="1:10" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A128" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B128" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E128" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="J124" s="20" t="s">
+      <c r="J128" s="20" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="125" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A125" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B125" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J125" s="20" t="s">
+    <row r="129" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A129" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B129" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J129" s="20" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="126" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A126" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B126" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J126" s="20" t="s">
+    <row r="130" spans="1:10" s="19" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A130" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B130" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J130" s="20" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="127" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A127" s="10" t="s">
+    <row r="131" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A131" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="J127" s="12" t="s">
+      <c r="J131" s="12" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A128" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B128" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C128" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="J128" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A129" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B129" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J129" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A130" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B130" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J130" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A131" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B131" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J131" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="C132" s="1" t="s">
+        <v>153</v>
+      </c>
       <c r="J132" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>149</v>
       </c>
@@ -2427,80 +2427,92 @@
         <v>40</v>
       </c>
       <c r="J133" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F134" s="1" t="s">
+      <c r="J134" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A135" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J135" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A136" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J136" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A137" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J137" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A138" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F138" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="J134" s="2" t="s">
+      <c r="J138" s="2" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="135" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A135" s="10" t="s">
+    <row r="139" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A139" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="J135" s="12" t="s">
+      <c r="J139" s="12" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A136" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="E136" s="7" t="b">
+    <row r="140" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A140" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E140" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="J136" s="8" t="s">
+      <c r="J140" s="8" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A137" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J137" s="8" t="s">
+    <row r="141" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A141" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J141" s="8" t="s">
         <v>94</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A138" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J138" s="8" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A139" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J139" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A140" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J140" s="8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A141" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="J141" s="8" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="34" x14ac:dyDescent="0.2">
@@ -2508,90 +2520,78 @@
         <v>138</v>
       </c>
       <c r="J142" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A143" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J143" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A144" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J144" s="8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A145" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J145" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A146" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J146" s="8" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="143" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A143" s="10" t="s">
+    <row r="147" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A147" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="J143" s="12" t="s">
+      <c r="J147" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="144" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A144" s="15" t="s">
+    <row r="148" spans="1:10" s="15" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A148" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="B144" s="15" t="s">
+      <c r="B148" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="C144" s="15" t="s">
+      <c r="C148" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="D144" s="15" t="b">
+      <c r="D148" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="I144" s="15" t="s">
+      <c r="I148" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="J144" s="16" t="s">
+      <c r="J148" s="16" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="145" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A145" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B145" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J145" s="18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="146" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A146" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B146" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J146" s="18" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="147" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A147" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B147" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J147" s="18" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="148" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A148" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="J148" s="12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="149" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A149" s="17" t="s">
         <v>138</v>
       </c>
       <c r="B149" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="E149" s="17" t="b">
-        <v>1</v>
-      </c>
       <c r="J149" s="18" t="s">
-        <v>162</v>
+        <v>104</v>
       </c>
     </row>
     <row r="150" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2602,10 +2602,10 @@
         <v>101</v>
       </c>
       <c r="J150" s="18" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="151" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A151" s="17" t="s">
         <v>138</v>
       </c>
@@ -2613,32 +2613,32 @@
         <v>101</v>
       </c>
       <c r="J151" s="18" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="152" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A152" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B152" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J152" s="18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="153" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A152" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="J152" s="12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A153" s="17" t="s">
         <v>138</v>
       </c>
       <c r="B153" s="17" t="s">
         <v>101</v>
       </c>
+      <c r="E153" s="17" t="b">
+        <v>1</v>
+      </c>
       <c r="J153" s="18" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="154" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A154" s="17" t="s">
         <v>138</v>
       </c>
@@ -2646,10 +2646,10 @@
         <v>101</v>
       </c>
       <c r="J154" s="18" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="155" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A155" s="17" t="s">
         <v>138</v>
       </c>
@@ -2657,23 +2657,67 @@
         <v>101</v>
       </c>
       <c r="J155" s="18" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="156" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A156" s="17" t="s">
         <v>138</v>
       </c>
       <c r="B156" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F156" s="17" t="s">
+      <c r="J156" s="18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A157" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B157" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J157" s="18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A158" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B158" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J158" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" s="17" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A159" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B159" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J159" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" s="17" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A160" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B160" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F160" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="H156" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="J156" s="18" t="s">
+      <c r="H160" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="J160" s="18" t="s">
         <v>120</v>
       </c>
     </row>

</xml_diff>